<commit_message>
Refresh timetable data (Jun 22-30) and auto-discover docx files
Replace the old Jun 8-16 source sheets with the new Jun 22-30 set and
reload the database from them.

parse-docx.js no longer hardcodes the filename->date map; it discovers
every "<WEEKDAY> <DD>.docx" in data/ and resolves each date by matching
the weekday against the calendar (anchored to Jun 2026, overridable via
IMPORT_YEAR/IMPORT_MONTH), so future sheets can be dropped in without
code changes.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TUTORS & MODULE.xlsx
+++ b/TUTORS & MODULE.xlsx
@@ -146,32 +146,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="6">
+  <fonts count="3">
     <font>
       <b val="0"/>
       <i val="0"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
-      <color rgb="FF980000"/>
-      <name val="Arial"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="0"/>
-      <i val="0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
@@ -201,36 +180,22 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
     </border>
-    <border>
-      <left>
-        <color rgb="FF000000"/>
-      </left>
-      <right>
-        <color rgb="FF000000"/>
-      </right>
-      <top>
-        <color rgb="FF000000"/>
-      </top>
-      <bottom>
-        <color rgb="FF000000"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="1" applyAlignment="1"/>
   </cellStyleXfs>
   <cellXfs count="4">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -489,7 +454,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{884143ED-B47A-4F89-A06D-167ACD3ECE3F}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{81CD18D6-A883-411C-B17E-0D37A8C06DCB}" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -946,7 +911,7 @@
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>
@@ -956,7 +921,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{83D2E5BD-5DC6-4EE3-98A4-58617D1B2B5E}" mc:Ignorable="x14ac xr xr2 xr3">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xr:uid="{8A623A9F-456D-42A5-B8EA-2308C0A91EC0}" mc:Ignorable="x14ac xr xr2 xr3">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -999,7 +964,7 @@
   </sheetData>
   <printOptions/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="portrait"/>
+  <pageSetup paperSize="1" pageOrder="downThenOver" orientation="portrait"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;C&amp;R</oddHeader>
     <oddFooter>&amp;L&amp;C&amp;R</oddFooter>

</xml_diff>